<commit_message>
fix logika perhitungan analisa pada output laporan excel
</commit_message>
<xml_diff>
--- a/Laporan_Analisa_Waste_Management_OktNov.xlsx
+++ b/Laporan_Analisa_Waste_Management_OktNov.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Downloads\SPIL\Waste Management\Analisa Waste Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD1B570-4F44-4DC6-A87E-95C7FCB20ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11546C8C-0C46-42AE-8325-93A96A0D6A8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ringkasan Executive" sheetId="1" r:id="rId1"/>
@@ -20,17 +20,12 @@
     <sheet name="Detail Eksternal" sheetId="5" r:id="rId5"/>
     <sheet name="Analisa Lanjutan" sheetId="6" r:id="rId6"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Detail BBM'!$A$1:$O$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Detail Eksternal'!$A$1:$K$44</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detail Internal'!$A$1:$T$123</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="194">
   <si>
     <t>RINGKASAN EXECUTIVE (OKT - NOV 2025)</t>
   </si>
@@ -72,9 +67,6 @@
   </si>
   <si>
     <t>Retribusi</t>
-  </si>
-  <si>
-    <t>Debit</t>
   </si>
   <si>
     <t>KOREKSI (Data 30 Sept)</t>
@@ -112,6 +104,9 @@
   </si>
   <si>
     <t>Brt Bersih</t>
+  </si>
+  <si>
+    <t>Debit</t>
   </si>
   <si>
     <t>BS</t>
@@ -979,7 +974,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47.140625" bestFit="1" customWidth="1"/>
@@ -1016,13 +1011,13 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <v>18919168</v>
+        <v>10919168</v>
       </c>
       <c r="C3">
         <v>110010</v>
       </c>
       <c r="D3">
-        <v>171.97680210889919</v>
+        <v>99.256140350877189</v>
       </c>
       <c r="E3">
         <v>122</v>
@@ -1095,7 +1090,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>8000000</v>
+        <v>-56500</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -1103,7 +1098,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>-56500</v>
+        <v>6218668</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1111,7 +1106,7 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>6218668</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -1119,15 +1114,7 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B18">
-        <v>18919168</v>
+        <v>10919168</v>
       </c>
     </row>
   </sheetData>
@@ -1143,13 +1130,11 @@
     <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14.28515625" bestFit="1" customWidth="1"/>
@@ -1159,31 +1144,31 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>10</v>
@@ -1248,7 +1233,7 @@
         <v>35</v>
       </c>
       <c r="P2">
-        <v>1534500</v>
+        <v>534500</v>
       </c>
       <c r="Q2" t="s">
         <v>36</v>
@@ -1908,7 +1893,7 @@
         <v>53</v>
       </c>
       <c r="P14">
-        <v>1463500</v>
+        <v>463500</v>
       </c>
       <c r="Q14" t="s">
         <v>36</v>
@@ -2621,7 +2606,7 @@
         <v>58</v>
       </c>
       <c r="P27">
-        <v>1786000</v>
+        <v>786000</v>
       </c>
       <c r="Q27" t="s">
         <v>36</v>
@@ -3505,7 +3490,7 @@
         <v>61</v>
       </c>
       <c r="P43">
-        <v>1977000</v>
+        <v>977000</v>
       </c>
       <c r="Q43" t="s">
         <v>36</v>
@@ -4884,7 +4869,7 @@
         <v>70</v>
       </c>
       <c r="P68">
-        <v>1495000</v>
+        <v>495000</v>
       </c>
       <c r="Q68" t="s">
         <v>36</v>
@@ -5647,7 +5632,7 @@
         <v>77</v>
       </c>
       <c r="P82">
-        <v>1513500</v>
+        <v>513500</v>
       </c>
       <c r="Q82" t="s">
         <v>36</v>
@@ -6475,7 +6460,7 @@
         <v>79</v>
       </c>
       <c r="P97">
-        <v>1439000</v>
+        <v>439000</v>
       </c>
       <c r="Q97" t="s">
         <v>36</v>
@@ -7191,7 +7176,7 @@
         <v>81</v>
       </c>
       <c r="P110">
-        <v>1548500</v>
+        <v>548500</v>
       </c>
       <c r="Q110" t="s">
         <v>36</v>
@@ -7935,7 +7920,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T123" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7945,6 +7929,7 @@
   <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="12.42578125" bestFit="1" customWidth="1"/>
@@ -8706,7 +8691,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O16" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8715,6 +8699,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -8776,11 +8769,9 @@
   <dimension ref="A1:K44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="16.28515625" bestFit="1" customWidth="1"/>
@@ -10252,7 +10243,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K44" xr:uid="{00000000-0001-0000-0400-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10261,6 +10251,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="46.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -10371,7 +10365,7 @@
         <v>33</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>